<commit_message>
add_fastq_information.py: add option to supply location of fastq files
</commit_message>
<xml_diff>
--- a/reportable_WWPilot_2026-03-04_AW.xlsx
+++ b/reportable_WWPilot_2026-03-04_AW.xlsx
@@ -838,196 +838,196 @@
     <t>CDPH-CLS-Genomics Center</t>
   </si>
   <si>
-    <t>26WBE-0663_S1_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0664_S2_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0665_S3_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0674_S5_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0676_S6_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0677_S7_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0681_S9_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0687_S10_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0690_S11_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0691_S13_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0692_S14_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0693_S15_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0695_S16_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0696_S17_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0697_S18_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0698_S19_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0699_S20_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0700_S21_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0701_S22_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0704_S24_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0705_S25_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0709_S26_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0712_S27_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0715_S29_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0716_S30_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0717_S31_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0718_S32_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0719_S33_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0720_S34_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0721_S35_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0722_S36_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0723_S37_R1_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0663_S1_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0664_S2_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0665_S3_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0674_S5_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0676_S6_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0677_S7_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0681_S9_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0687_S10_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0690_S11_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0691_S13_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0692_S14_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0693_S15_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0695_S16_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0696_S17_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0697_S18_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0698_S19_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0699_S20_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0700_S21_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0701_S22_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0704_S24_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0705_S25_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0709_S26_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0712_S27_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0715_S29_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0716_S30_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0717_S31_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0718_S32_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0719_S33_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0720_S34_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0721_S35_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0722_S36_R2_001.fastq.gz</t>
-  </si>
-  <si>
-    <t>26WBE-0723_S37_R2_001.fastq.gz</t>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0663_S1_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0664_S2_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0665_S3_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0674_S5_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0676_S6_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0677_S7_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0681_S9_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0687_S10_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0690_S11_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0691_S13_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0692_S14_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0693_S15_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0695_S16_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0696_S17_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0697_S18_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0698_S19_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0699_S20_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0700_S21_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0701_S22_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0704_S24_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0705_S25_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0709_S26_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0712_S27_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0715_S29_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0716_S30_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0717_S31_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0718_S32_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0719_S33_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0720_S34_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0721_S35_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0722_S36_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0723_S37_R1_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0663_S1_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0664_S2_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0665_S3_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0674_S5_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0676_S6_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0677_S7_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0681_S9_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0687_S10_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0690_S11_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0691_S13_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0692_S14_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0693_S15_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0695_S16_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0696_S17_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0697_S18_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0698_S19_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0699_S20_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0700_S21_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0701_S22_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0704_S24_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0705_S25_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0709_S26_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0712_S27_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0715_S29_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0716_S30_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0717_S31_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0718_S32_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0719_S33_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0720_S34_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0721_S35_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0722_S36_R2_001.fastq.gz</t>
+  </si>
+  <si>
+    <t>/home/dbest/Analysis/Covid19/CovidSeq/WWPilot_2026-03-04_AW/untrimmed/26WBE-0723_S37_R2_001.fastq.gz</t>
   </si>
   <si>
     <t>paired</t>

</xml_diff>